<commit_message>
Update 深川鐵板蓋飯 with official menu poster
</commit_message>
<xml_diff>
--- a/彰化市大埔商圈59家精選店家完整名冊.xlsx
+++ b/彰化市大埔商圈59家精選店家完整名冊.xlsx
@@ -2638,17 +2638,17 @@
       </c>
       <c r="I39" s="12" t="inlineStr">
         <is>
-          <t>大火現炒鐵板肉片 ‧ 附荷包蛋高CP值蓋飯</t>
+          <t>餐餐皆附荷包蛋 ‧ 買5碗送荷包蛋或起司二選一</t>
         </is>
       </c>
       <c r="J39" s="12" t="inlineStr">
         <is>
-          <t>招牌鐵板牛肉蓋飯(附蛋)、人氣鐵板豬肉蓋飯、巨飽雙拼雙份肉蓋飯、韓式泡菜牛肉蓋飯、現炒鐵板高麗菜/杏鮑菇</t>
+          <t>鐵板牛肉蓋飯(附荷包蛋)、泡菜牛肉蓋飯 / 泡菜豬肉蓋飯、巨飽雙倍肉系列 (牛/豬/雞)、牛+雞/牛+豬雙拼蓋飯、九層塔蛋 / 起司蛋 / 炒時蔬</t>
         </is>
       </c>
       <c r="K39" s="12" t="inlineStr">
         <is>
-          <t>大埔路超人氣鐵板風味蓋飯！將現點現炒的大火鑊氣鐵板燒料理融入豐盛蓋飯中，招牌鐵板牛肉與豬肉蓋飯均附金黃荷包蛋，肉質鮮嫩醬汁入味超下飯，更有雙份肉量巨飽系列與炒時蔬，是在地學生與上班族午晚餐高CP值首選！</t>
+          <t>大埔路超人氣鐵板風味蓋飯！餐點皆附金黃荷包蛋，提供鐵板牛肉/豬肉/雞肉、特製泡菜系列、大肉量巨飽系列與雙拼組合。更有自取買5碗或外送買10碗送荷包蛋/起司二選一好康，自備環保餐盒享加碼優惠！</t>
         </is>
       </c>
       <c r="L39" s="13" t="inlineStr">

</xml_diff>